<commit_message>
fix(pricing): the monadic half of H5, one bootstrap policy, and two first-contact defaults
The review named the monadic intent line beside the Gabor-Granger one and
the first commit fixed only the latter: 1 = Yes / 2 = No intent still read
as 100% in every cell. Now a declared-binary intent column is checked, with
Binary_Coding = ONE_TWO on the Monadic sheet. The monadic bootstrap resampled
with weighted probabilities and then fitted with the weights, counting them
twice; it now resamples with equal probability carrying the weights, the
same policy as the other two. Generate_Tabs_Export and Export_WTP refuse on
Y until the exporter exists, rather than passing in silence. The GUI stats
pack checkbox defaults to on, since it is now authoritative and stats packs
are contractual. Suite 997 / 0 / 0 / 14 warnings.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/pricing/docs/templates/Pricing_Config_Template.xlsx
+++ b/modules/pricing/docs/templates/Pricing_Config_Template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="301">
   <si>
     <t xml:space="preserve">TURAS Pricing Module - Configuration</t>
   </si>
@@ -214,7 +214,7 @@
     <t xml:space="preserve">N</t>
   </si>
   <si>
-    <t xml:space="preserve">Write {output}_tabs_pricing.xlsx: the Gabor-Granger acceptance grid as 0/1 columns a tabs (crosstab) project can read as a Multi_Mention question, with a QuestionMap snippet and a METHOD sheet. Needs ID_Variable.</t>
+    <t xml:space="preserve">Write {output}_tabs_pricing.xlsx: the Gabor-Granger acceptance grid as 0/1 columns a tabs (crosstab) project can read as a Multi_Mention question, with a QuestionMap snippet and a METHOD sheet. Needs ID_Variable. Not built yet: Y refuses until the pricing v2 session lands.</t>
   </si>
   <si>
     <t xml:space="preserve">Tabs_Question_Code</t>
@@ -232,7 +232,7 @@
     <t xml:space="preserve">Export_WTP</t>
   </si>
   <si>
-    <t xml:space="preserve">Also export a per-respondent willingness-to-pay column (midpoint of the Van Westendorp cheap and expensive answers), stamped as derived on the METHOD sheet.</t>
+    <t xml:space="preserve">Also export a per-respondent willingness-to-pay column (midpoint of the Van Westendorp cheap and expensive answers), stamped as derived on the METHOD sheet. Not built yet: Y refuses until the pricing v2 session lands.</t>
   </si>
   <si>
     <t xml:space="preserve">MONOTONICITY HANDLING</t>
@@ -653,6 +653,9 @@
   </si>
   <si>
     <t xml:space="preserve">Integer on intent scale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For Intent_Type = binary: ZERO_ONE means 1 = would buy, 0 = would not. ONE_TWO means 1 = would buy, 2 = would not (the usual survey export). Any other value refuses.</t>
   </si>
   <si>
     <t xml:space="preserve">MODEL SETTINGS</t>
@@ -3059,113 +3062,130 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
+      <c r="E11" s="14" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>215</v>
-      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="E13" s="14" t="s">
         <v>216</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="E14" s="14" t="s">
         <v>220</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>221</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>48</v>
+        <v>222</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>50</v>
+        <v>224</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>153</v>
+        <v>48</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>155</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B18" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="C17" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D17" s="13" t="s">
+      <c r="C18" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="E18" s="14" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3174,22 +3194,22 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B10">
       <formula1>1</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B13:B13">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:B14">
       <formula1>10</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:B14">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B15:B15">
       <formula1>50</formula1>
       <formula2>500</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B16:B16">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B17">
       <formula1>500</formula1>
       <formula2>10000</formula2>
     </dataValidation>
@@ -3198,7 +3218,7 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"binary,scale"</xm:f>
@@ -3207,21 +3227,27 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
+            <xm:f>"ZERO_ONE,ONE_TWO"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B11:B11</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
             <xm:f>"logistic,log_logistic"</xm:f>
           </x14:formula1>
-          <xm:sqref>B12:B12</xm:sqref>
+          <xm:sqref>B13:B13</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B15:B15</xm:sqref>
+          <xm:sqref>B16:B16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"0.90,0.95,0.99"</xm:f>
           </x14:formula1>
-          <xm:sqref>B17:B17</xm:sqref>
+          <xm:sqref>B18:B18</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3244,29 +3270,29 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>10</v>
@@ -3274,27 +3300,27 @@
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B5" s="17" t="n">
         <v>9.99</v>
@@ -3309,12 +3335,12 @@
         <v>23</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>12.99</v>
@@ -3329,12 +3355,12 @@
         <v>23</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>16.99</v>
@@ -3349,7 +3375,7 @@
         <v>23</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -3462,12 +3488,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3">
@@ -3506,7 +3532,7 @@
     </row>
     <row r="6">
       <c r="A6" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -3515,70 +3541,70 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -3621,23 +3647,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5">
@@ -3645,7 +3671,7 @@
         <v>23</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6">
@@ -3653,7 +3679,7 @@
         <v>23</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7">
@@ -3661,7 +3687,7 @@
         <v>23</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8">
@@ -3669,15 +3695,15 @@
         <v>23</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="10">
@@ -3685,7 +3711,7 @@
         <v>23</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11">
@@ -3693,7 +3719,7 @@
         <v>23</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12">
@@ -3701,15 +3727,15 @@
         <v>23</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14">
@@ -3717,7 +3743,7 @@
         <v>23</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15">
@@ -3725,7 +3751,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16">
@@ -3733,15 +3759,15 @@
         <v>23</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18">
@@ -3749,7 +3775,7 @@
         <v>23</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19">
@@ -3757,7 +3783,7 @@
         <v>23</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="20">
@@ -3765,7 +3791,7 @@
         <v>23</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="21">
@@ -3773,7 +3799,7 @@
         <v>23</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -3792,15 +3818,15 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>23</v>
@@ -3816,7 +3842,7 @@
     </row>
     <row r="4">
       <c r="A4" s="13" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>23</v>
@@ -3824,7 +3850,7 @@
     </row>
     <row r="5">
       <c r="A5" s="13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>23</v>
@@ -3832,7 +3858,7 @@
     </row>
     <row r="6">
       <c r="A6" s="13" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>23</v>
@@ -3840,7 +3866,7 @@
     </row>
     <row r="7">
       <c r="A7" s="13" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>23</v>
@@ -3848,7 +3874,7 @@
     </row>
     <row r="8">
       <c r="A8" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>23</v>
@@ -3873,24 +3899,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C2" s="13" t="s">
         <v>23</v>

</xml_diff>